<commit_message>
data-cleanup: minor nutrition input fixes
Notes-column terminology rewords ('smd used' / 'n not available so smd used' -> '"n not available, d used"') in 4 CSVs (Caffeine/shen2019, Creatine/lanhers2015 leg press + squat, Creatine/lanhers2017 chest_strength_excl); a 'SMD'->'d' header rename + new empty 'notes' column with one annotation in VitaminD/stockton2011; and workbook-cleanup XLSX size reductions in 7 extraction workbooks. No g/se_g/d/se_d numeric values changed, no row counts changed, no analysis-ready shape changed. The Commit 5 v4 sidecars remain aligned: the loader resolves g/se_g first (.resolve_effect_input in 00_utils.R) and ignores notes; the stockton2011 'SMD'->'d' rename affects only the unused d/se_d fallback. Two XLSX files (Creatine/doma2022 48h_post_protocol and Omega3/kong2025 depression) are extraction workbooks with no companion analysis-ready CSV; workbook cleanup only.
</commit_message>
<xml_diff>
--- a/data/Omega3/kong2025/kong2025_omega3_depression.xlsx
+++ b/data/Omega3/kong2025/kong2025_omega3_depression.xlsx
@@ -44,7 +44,7 @@
     <t>Year</t>
   </si>
   <si>
-    <t>SMD</t>
+    <t>d</t>
   </si>
   <si>
     <t>lCI</t>
@@ -188,7 +188,7 @@
     <t>notes</t>
   </si>
   <si>
-    <t>n not available, smd used</t>
+    <t>n not available, d used</t>
   </si>
 </sst>
 </file>

</xml_diff>